<commit_message>
merged-cells: simplify test file to ease debugging
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Excell_T2_small.xlsx
+++ b/Ref_Files/Test_Excell_T2_small.xlsx
@@ -11,7 +11,7 @@
     <sheet name="КСС_ОП1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">КСС_ОП1!$A$7</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">КСС_ОП1!$A$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,19 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="34">
-  <si>
-    <t xml:space="preserve">Тест</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Някаква информация</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Някакво по-дълго описание на поставената задача. Може да съдържа няколко реда …</t>
-  </si>
-  <si>
-    <t xml:space="preserve">КОЛИЧЕСТВЕНО - СТОЙНОСТНА СМЕТКА (КСС)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
   <si>
     <t xml:space="preserve">№ по ред</t>
   </si>
@@ -136,47 +124,15 @@
   <si>
     <t xml:space="preserve">III.</t>
   </si>
-  <si>
-    <t xml:space="preserve">IV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 6:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XIV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 18:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ В ЕВРО БЕЗ ДДС (I+II+III+IV+V+VI+VII+VIII+IX+X+XI+XII+XIII+XIV):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XVI.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДДС 20 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XVII.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩО ВСИЧКО В ЕВРО С ДДС (XV+XVI):</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,46 +158,6 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Verdana"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
@@ -305,7 +221,7 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -321,7 +237,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8EFD8"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFEAF1CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -336,32 +252,8 @@
         <bgColor rgb="FFF8EFD8"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.3999"/>
-        <bgColor rgb="FFCCCCFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.7999"/>
-        <bgColor rgb="FFF8EFD8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.5999"/>
-        <bgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.3999"/>
-        <bgColor rgb="FFFFE699"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -370,50 +262,8 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
       <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="thin"/>
-      <top style="medium"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
-      <top style="medium"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right style="medium"/>
-      <top style="medium"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
       <top style="thin"/>
       <bottom style="thin"/>
       <diagonal/>
@@ -444,7 +294,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -453,179 +303,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -641,7 +367,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFF8EFD8"/>
+      <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -658,7 +384,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFF8EFD8"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -675,11 +401,11 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFEAF1CD"/>
-      <rgbColor rgb="FFFFE699"/>
-      <rgbColor rgb="FF9DC3E6"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFD966"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -890,429 +616,298 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="8" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="6" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-    </row>
-    <row r="2" s="8" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-    </row>
-    <row r="3" s="8" customFormat="true" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-    </row>
-    <row r="4" s="8" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-    </row>
-    <row r="5" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="15"/>
-    </row>
-    <row r="6" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <f aca="false">D4*1</f>
+        <v>1</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="18" t="s">
+      <c r="A7" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>222</v>
+      </c>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>222</v>
+      </c>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="C10" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+      <c r="D10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B11" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="25" t="n">
+      <c r="C12" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="9" t="n">
         <f aca="false">D10*1</f>
         <v>1</v>
       </c>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="27" t="n">
+      <c r="A13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="29" t="n">
+      <c r="B16" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="13" t="n">
         <v>222</v>
       </c>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="29" t="n">
-        <v>222</v>
-      </c>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="14"/>
+      <c r="M17" s="14"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" s="25" t="n">
-        <f aca="false">D16*1</f>
-        <v>1</v>
-      </c>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="D20" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C21" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="D21" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-    </row>
-    <row r="22" s="30" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="B22" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="D22" s="29" t="n">
-        <v>222</v>
-      </c>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="32"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="33"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34" t="s">
-        <v>26</v>
-      </c>
-      <c r="B24" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="36"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="B25" s="38" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="30"/>
-      <c r="J25" s="30"/>
-      <c r="K25" s="30"/>
-      <c r="L25" s="30"/>
-      <c r="M25" s="30"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="40" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="41"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="42"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="30"/>
-      <c r="K26" s="30"/>
-      <c r="L26" s="30"/>
-      <c r="M26" s="30"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="43" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" s="44"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="45"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="30"/>
-      <c r="B28" s="30"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="30"/>
-      <c r="K28" s="30"/>
-      <c r="L28" s="30"/>
-      <c r="M28" s="30"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="30"/>
-      <c r="B29" s="30"/>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="30"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-    </row>
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+    </row>
+    <row r="1048104" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048105" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048106" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048107" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048108" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048109" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048110" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048111" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048112" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048113" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048114" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048115" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048116" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048117" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1764,29 +1359,20 @@
     <row r="1048563" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048565" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="1">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B27:E27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
merged-cells: totally simplify test
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Excell_T2_small.xlsx
+++ b/Ref_Files/Test_Excell_T2_small.xlsx
@@ -11,7 +11,7 @@
     <sheet name="КСС_ОП1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">КСС_ОП1!$A$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">#REF!</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,34 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
-  <si>
-    <t xml:space="preserve">№ по ред</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Наименование на работите</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ед. мярка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Колич.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ед. цена</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Стойност</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сецкия 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Строителна част</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="6">
   <si>
     <t xml:space="preserve">Операция Х-00700</t>
   </si>
@@ -69,61 +42,6 @@
   <si>
     <t xml:space="preserve">Операция Х-00702</t>
   </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00200</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">m</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">II.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">m</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">III.</t>
-  </si>
 </sst>
 </file>
 
@@ -132,7 +50,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,22 +81,6 @@
       <charset val="204"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -201,27 +103,12 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <vertAlign val="superscript"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -230,26 +117,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDEB340"/>
-        <bgColor rgb="FFFF9900"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8EFD8"/>
-        <bgColor rgb="FFEAF1CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFC0D66A"/>
-        <bgColor rgb="FFDEB340"/>
+        <bgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEAF1CD"/>
-        <bgColor rgb="FFF8EFD8"/>
+        <bgColor rgb="FFCCFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -294,7 +169,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -303,55 +178,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -384,7 +227,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF8EFD8"/>
+      <rgbColor rgb="FFEAF1CD"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -400,7 +243,7 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFEAF1CD"/>
+      <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -409,7 +252,7 @@
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFDEB340"/>
+      <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
@@ -617,286 +460,173 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
+        <v>5</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <f aca="false">D1*1</f>
+        <v>1</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="9" t="n">
+      <c r="A6" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4" t="n">
         <f aca="false">D4*1</f>
         <v>1</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="13" t="n">
-        <v>222</v>
-      </c>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="13" t="n">
-        <v>222</v>
-      </c>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <f aca="false">D10*1</f>
-        <v>1</v>
-      </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-    </row>
-    <row r="16" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>222</v>
-      </c>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="14"/>
-    </row>
+    <row r="1048096" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048097" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048098" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048099" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048100" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048101" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048102" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048103" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048104" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048105" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048106" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1359,9 +1089,9 @@
     <row r="1048563" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048565" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1371,9 +1101,6 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
merged-cells: extended test file
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Excell_T2_small.xlsx
+++ b/Ref_Files/Test_Excell_T2_small.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="8">
   <si>
     <t xml:space="preserve">Операция Х-00700</t>
   </si>
@@ -42,6 +42,12 @@
   <si>
     <t xml:space="preserve">Операция Х-00702</t>
   </si>
+  <si>
+    <t xml:space="preserve">Операция Х-00704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Операция Х-00703</t>
+  </si>
 </sst>
 </file>
 
@@ -50,7 +56,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -100,12 +106,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
     </font>
   </fonts>
   <fills count="4">
@@ -169,7 +169,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -192,10 +192,6 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -447,7 +443,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M1048576"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
@@ -590,34 +586,84 @@
       <c r="F8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
+      <c r="A9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
+      <c r="A10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
     </row>
     <row r="1048096" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048097" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>